<commit_message>
Mise à jour automatique des prix Donner
</commit_message>
<xml_diff>
--- a/Prix_Donner_TTC.xlsx
+++ b/Prix_Donner_TTC.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B526"/>
+  <dimension ref="A1:B528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1717,7 +1717,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Donner Go ampli guitare Noir</t>
+          <t>Donner Go ampli guitare - Donner Go【Noir】</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -1727,137 +1727,137 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Donner Starryctrl Contrôleur MIDI, Noir</t>
+          <t>Donner Go ampli guitare - Donner Go II【Noir】</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>69.98999999999999</v>
+        <v>129.99</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>【Donner】Pour la différence de prix</t>
+          <t>Donner Go ampli guitare - Donner Go II【Blanc】</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>180</v>
+        <v>129.99</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano</t>
+          <t>Donner Starryctrl Contrôleur MIDI, Noir</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>469.99</v>
+        <v>69.98999999999999</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano + noir</t>
+          <t>【Donner】Pour la différence de prix</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>539.98</v>
+        <v>180</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano + banc (match officiel)</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>559.98</v>
+        <v>469.99</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano + noir</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>579.98</v>
+        <v>539.98</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano + banc (match officiel)</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>399.99</v>
+        <v>559.98</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + noir</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>485.98</v>
+        <v>579.98</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + banc (match officiel)</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>489.98</v>
+        <v>399.99</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + noir</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>509.98</v>
+        <v>485.98</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Donner CV-3 Système de monitoring intra-auriculaire sans fil</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + banc (match officiel)</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>159.99</v>
+        <v>489.98</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - Sunburst</t>
+          <t>Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>209.99</v>
+        <v>509.98</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - naturel</t>
+          <t>Donner CV-3 Système de monitoring intra-auriculaire sans fil</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>209.99</v>
+        <v>159.99</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - Noir</t>
+          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - Sunburst</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -1867,7 +1867,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - Blanc</t>
+          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - naturel</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -1877,117 +1877,117 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Donner DED-200X Batterie Électronique - 5 Tambours et 4 Cymbales</t>
+          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - Noir</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>499.99</v>
+        <v>209.99</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Donner DED-200X Batterie Électronique - Nouvelle 5 Tambours et 4 Cymbales</t>
+          <t>【Boîte ouverte】Donner HUSH X Guitare Électrique Sans Tête - Blanc</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>599.99</v>
+        <v>209.99</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Donner DED-200X Batterie Électronique - 5 Tambours et 3 Cymbales</t>
+          <t>Donner DED-200X Batterie Électronique - 5 Tambours et 4 Cymbales</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>589.99</v>
+        <v>499.99</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Donner Beat Go Kit de batterie électronique portable</t>
+          <t>Donner DED-200X Batterie Électronique - Nouvelle 5 Tambours et 4 Cymbales</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>289.99</v>
+        <v>599.99</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Donner Tabouret De Piano À Hauteur Réglable - Blanc mat</t>
+          <t>Donner DED-200X Batterie Électronique - 5 Tambours et 3 Cymbales</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>119.99</v>
+        <v>589.99</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Donner Tabouret De Piano À Hauteur Réglable - Beige mat</t>
+          <t>Donner Beat Go Kit de batterie électronique portable</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>119.99</v>
+        <v>289.99</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Donner Table de percussion</t>
+          <t>Donner Tabouret De Piano À Hauteur Réglable - Blanc mat</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>39.99</v>
+        <v>119.99</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano</t>
+          <t>Donner Tabouret De Piano À Hauteur Réglable - Beige mat</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>599.99</v>
+        <v>119.99</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc【Pack Officiel】</t>
+          <t>Donner Table de percussion</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>699.99</v>
+        <v>39.99</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc</t>
+          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>699.99</v>
+        <v>599.99</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano</t>
+          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc【Pack Officiel】</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>599.99</v>
+        <v>699.99</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc【Pack Officiel】</t>
+          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -1997,637 +1997,637 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc</t>
+          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>699.99</v>
+        <v>599.99</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 32 Touches Bleu clair</t>
+          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc【Pack Officiel】</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>69.98999999999999</v>
+        <v>699.99</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 32 Touches Rose clair</t>
+          <t>【Boîte ouverte】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>69.98999999999999</v>
+        <v>699.99</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 44 Touches avec Support Bleu clair</t>
+          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 32 Touches Bleu clair</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>89.98999999999999</v>
+        <v>69.98999999999999</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 44 Touches avec Support Rose clair</t>
+          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 32 Touches Rose clair</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>89.98999999999999</v>
+        <v>69.98999999999999</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Donner DED-70L Batterie électronique Avec Lumière LED</t>
+          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 44 Touches avec Support Bleu clair</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>269.99</v>
+        <v>89.98999999999999</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Donner Starrykey-37 Play Contrôleur MIDI</t>
+          <t>【Déstockage】Eastar KIDO Miniature Clavier Numérique - 44 Touches avec Support Rose clair</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>149.99</v>
+        <v>89.98999999999999</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Donner DDA-20SE Enceinte de monitoring de batterie</t>
+          <t>Donner DED-70L Batterie électronique Avec Lumière LED</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>129.99</v>
+        <v>269.99</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano</t>
+          <t>Donner Starrykey-37 Play Contrôleur MIDI</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>339.99</v>
+        <v>149.99</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco de Piano Noir</t>
+          <t>Donner DDA-20SE Enceinte de monitoring de batterie</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>479.98</v>
+        <v>129.99</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banc réglable X-Style</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>479.98</v>
+        <v>339.99</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco de Piano Noir</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>499.98</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco de Piano Noir + Tourneur de Page</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>539.97</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>539.97</v>
+        <v>499.98</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco + Tourneur de Page</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco de Piano Noir + Tourneur de Page</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>559.97</v>
+        <v>539.97</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>519.98</v>
+        <v>539.97</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - DDP-400 Piano</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Banco + Tourneur de Page</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>829.99</v>
+        <v>559.97</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano</t>
+          <t>Donner DDP-50 88 touches Lestées Piano numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>909.98</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano Blanc</t>
+          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - DDP-400 Piano</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>925.98</v>
+        <v>829.99</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Tourneur de Page</t>
+          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>899.98</v>
+        <v>909.98</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano Blanc</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>979.97</v>
+        <v>925.98</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano Blanc + Tourneur de Page</t>
+          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>995.97</v>
+        <v>899.98</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Eastar EDA-100 Digital Aerophone Noir</t>
+          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>122.99</v>
+        <v>979.97</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare</t>
+          <t>Donner DDP-400 Piano Numérique à Touches Pondérées - Piano + Banc de Piano Blanc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>299.99</v>
+        <v>995.97</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + JW Pédale</t>
+          <t>Eastar EDA-100 Digital Aerophone Noir</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>418.99</v>
+        <v>122.99</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + Pocket Go Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>419.98</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + DBM-100 Métronome Noir</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>369.98</v>
+        <v>418.99</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + DBM-100 Métronome Jaune</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>369.98</v>
+        <v>419.98</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + DBM-100 Métronome Noir</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>279.99</v>
+        <v>369.98</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + JW Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Bois naturel / Guitare + DBM-100 Métronome Jaune</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>418.99</v>
+        <v>369.98</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + Pocket Go Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>419.98</v>
+        <v>279.99</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + DBM-100 Métronome Noir</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>369.98</v>
+        <v>418.99</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + DBM-100 Métronome Jaune</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>369.98</v>
+        <v>419.98</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + DBM-100 Métronome Noir</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>299.99</v>
+        <v>369.98</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + JW Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Blanc / Guitare + DBM-100 Métronome Jaune</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>398.99</v>
+        <v>369.98</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + Pocket Go Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>399.98</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + DBM-100 Métronome Noir</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>352.98</v>
+        <v>398.99</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + DBM-100 Métronome Jaune</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>352.98</v>
+        <v>399.98</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + DBM-100 Métronome Noir</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>299.99</v>
+        <v>352.98</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + JW Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Rouge métallisé / Guitare + DBM-100 Métronome Jaune</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>398.99</v>
+        <v>352.98</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + Pocket Go Pédale</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>399.98</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + DBM-100 Métronome Noir</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>352.98</v>
+        <v>398.99</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + DBM-100 Métronome Jaune</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>352.98</v>
+        <v>399.98</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Donner DKS-200 Pied Réglable Pliable Pour Clavier Noir</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + DBM-100 Métronome Noir</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>99.98999999999999</v>
+        <v>352.98</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Donner Pocket Go Pédale Portable Multi Effets Guitare</t>
+          <t>Donner HLX-500 Guitare Électrique Moderne Sans Tête【ancienne réf. NHL-500】 - Sherwood Green / Guitare + DBM-100 Métronome Jaune</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>99.98999999999999</v>
+        <v>352.98</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Donner MAMP2 Puissant Amplificateur 2 Canaux</t>
+          <t>Donner DKS-200 Pied Réglable Pliable Pour Clavier Noir</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>126.99</v>
+        <v>99.98999999999999</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Donner Starrypad Mini-Contrôleur MIDI</t>
+          <t>Donner Pocket Go Pédale Portable Multi Effets Guitare</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>62.99</v>
+        <v>99.98999999999999</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Donner DBM-100 Métronome Accordeur 3-en-1 Rechargeable - Noir</t>
+          <t>Donner MAMP2 Puissant Amplificateur 2 Canaux</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>59.99</v>
+        <v>126.99</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Donner DBM-100 Métronome Accordeur 3-en-1 Rechargeable - Jaune</t>
+          <t>Donner Starrypad Mini-Contrôleur MIDI</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>56.99</v>
+        <v>62.99</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Donner DK-10S 61 Touches Clavier Électronique - clavier électronique</t>
+          <t>Donner DBM-100 Métronome Accordeur 3-en-1 Rechargeable - Noir</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>139.99</v>
+        <v>59.99</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Donner DK-10S 61 Touches Clavier Électronique - Clavier + Banc X-Style</t>
+          <t>Donner DBM-100 Métronome Accordeur 3-en-1 Rechargeable - Jaune</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>219.98</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Donner DK-10S 61 Touches Clavier Électronique - Clavier + Banc de Piano</t>
+          <t>Donner DK-10S 61 Touches Clavier Électronique - clavier électronique</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>219.98</v>
+        <v>139.99</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Donner Banquette Piano Duo Réglable avec Rangement</t>
+          <t>Donner DK-10S 61 Touches Clavier Électronique - Clavier + Banc X-Style</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>119.99</v>
+        <v>219.98</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Donner HUSH C Guitare Nylon Voyage Électro-Acoustique - Sunburst</t>
+          <t>Donner DK-10S 61 Touches Clavier Électronique - Clavier + Banc de Piano</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>284.99</v>
+        <v>219.98</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Donner HUSH C Guitare Nylon Voyage Électro-Acoustique - Noir</t>
+          <t>Donner Banquette Piano Duo Réglable avec Rangement</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>284.99</v>
+        <v>119.99</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Donner Banquette Piano Duo Réglable Confort</t>
+          <t>Donner HUSH C Guitare Nylon Voyage Électro-Acoustique - Sunburst</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>115.99</v>
+        <v>284.99</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Donner M100 Casque de monitoring studio</t>
+          <t>Donner HUSH C Guitare Nylon Voyage Électro-Acoustique - Noir</t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>59.99</v>
+        <v>284.99</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Donner DEP-08 Piano Numérique - Piano</t>
+          <t>Donner Banquette Piano Duo Réglable Confort</t>
         </is>
       </c>
       <c r="B214" t="n">
-        <v>229.99</v>
+        <v>115.99</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Donner DEP-08 Piano Numérique - Piano + Banc réglable X-Style</t>
+          <t>Donner M100 Casque de monitoring studio</t>
         </is>
       </c>
       <c r="B215" t="n">
-        <v>359.98</v>
+        <v>59.99</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Donner DEP-08 Piano Numérique - Piano + banc</t>
+          <t>Donner DEP-08 Piano Numérique - Piano</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>359.98</v>
+        <v>229.99</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Donner DEP-1 Piano Numérique Portable - Piano</t>
+          <t>Donner DEP-08 Piano Numérique - Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B217" t="n">
-        <v>199.99</v>
+        <v>359.98</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Donner DEP-1 Piano Numérique Portable - Piano + banc</t>
+          <t>Donner DEP-08 Piano Numérique - Piano + banc</t>
         </is>
       </c>
       <c r="B218" t="n">
-        <v>299.98</v>
+        <v>359.98</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Donner DEP-1 Piano Numérique Portable - Piano + Support de clavier</t>
+          <t>Donner DEP-1 Piano Numérique Portable - Piano</t>
         </is>
       </c>
       <c r="B219" t="n">
-        <v>299.98</v>
+        <v>199.99</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Donner DEP-1 Piano Numérique Portable - Piano + Banc réglable X-Style</t>
+          <t>Donner DEP-1 Piano Numérique Portable - Piano + banc</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -2637,107 +2637,107 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Donner DEP-1 Piano Numérique Portable - Piano + Support de clavier + Banc X-Style</t>
+          <t>Donner DEP-1 Piano Numérique Portable - Piano + Support de clavier</t>
         </is>
       </c>
       <c r="B221" t="n">
-        <v>367.97</v>
+        <v>299.98</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Donner DEP-1 Piano Numérique Portable - Piano + Support de clavier + banc</t>
+          <t>Donner DEP-1 Piano Numérique Portable - Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B222" t="n">
-        <v>392.97</v>
+        <v>299.98</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Donner DED-70 Batterie Electronique</t>
+          <t>Donner DEP-1 Piano Numérique Portable - Piano + Support de clavier + Banc X-Style</t>
         </is>
       </c>
       <c r="B223" t="n">
-        <v>199.99</v>
+        <v>367.97</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Donner DED-80 Batterie électrique - Noir</t>
+          <t>Donner DEP-1 Piano Numérique Portable - Piano + Support de clavier + banc</t>
         </is>
       </c>
       <c r="B224" t="n">
-        <v>219.99</v>
+        <v>392.97</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Donner DED-80 Batterie électrique - Blanc</t>
+          <t>Donner DED-70 Batterie Electronique</t>
         </is>
       </c>
       <c r="B225" t="n">
-        <v>219.99</v>
+        <v>199.99</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Donner Essential L1 Synthétiseur - L1</t>
+          <t>Donner DED-80 Batterie électrique - Noir</t>
         </is>
       </c>
       <c r="B226" t="n">
-        <v>279.99</v>
+        <v>219.99</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Donner Essential L1 Synthétiseur - KB-32M</t>
+          <t>Donner DED-80 Batterie électrique - Blanc</t>
         </is>
       </c>
       <c r="B227" t="n">
-        <v>119.99</v>
+        <v>219.99</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Donner Essential L1 Synthétiseur - Pack</t>
+          <t>Donner Essential L1 Synthétiseur - L1</t>
         </is>
       </c>
       <c r="B228" t="n">
-        <v>399.98</v>
+        <v>279.99</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA S300 Domestique Piano Numérique - Piano+Banc【Forfait officiel】</t>
+          <t>Donner Essential L1 Synthétiseur - KB-32M</t>
         </is>
       </c>
       <c r="B229" t="n">
-        <v>799.99</v>
+        <v>119.99</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA S300 Domestique Piano Numérique - Piano+Banc</t>
+          <t>Donner Essential L1 Synthétiseur - Pack</t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>799.99</v>
+        <v>399.98</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA S300 Domestique Piano Numérique - Piano</t>
+          <t>【Piano + banc gratuit】Donner OURA S300 Domestique Piano Numérique - Piano+Banc【Forfait officiel】</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2747,157 +2747,157 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Donner OURA S100 Tabouret Bois Massif assorti (DKB-100)</t>
+          <t>【Piano + banc gratuit】Donner OURA S300 Domestique Piano Numérique - Piano+Banc</t>
         </is>
       </c>
       <c r="B232" t="n">
-        <v>102.99</v>
+        <v>799.99</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Noir Aurora / Guitare</t>
+          <t>【Piano + banc gratuit】Donner OURA S300 Domestique Piano Numérique - Piano</t>
         </is>
       </c>
       <c r="B233" t="n">
-        <v>409.99</v>
+        <v>799.99</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Noir Aurora / Guitare + JW Pédale</t>
+          <t>Donner OURA S100 Tabouret Bois Massif assorti (DKB-100)</t>
         </is>
       </c>
       <c r="B234" t="n">
-        <v>498.99</v>
+        <v>102.99</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Noir Aurora / Guitare + Pocket Go Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Noir Aurora / Guitare</t>
         </is>
       </c>
       <c r="B235" t="n">
-        <v>499.98</v>
+        <v>409.99</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Blanc-Or / Guitare</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Noir Aurora / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B236" t="n">
-        <v>409.99</v>
+        <v>498.99</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Blanc-Or / Guitare + JW Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Noir Aurora / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>498.99</v>
+        <v>499.98</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Blanc-Or / Guitare + Pocket Go Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Blanc-Or / Guitare</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>499.98</v>
+        <v>409.99</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Noir / Guitare</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Blanc-Or / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B239" t="n">
-        <v>399.99</v>
+        <v>498.99</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Noir / Guitare + JW Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Blanc-Or / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B240" t="n">
-        <v>498.99</v>
+        <v>499.98</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Noir / Guitare + Pocket Go Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Noir / Guitare</t>
         </is>
       </c>
       <c r="B241" t="n">
-        <v>499.98</v>
+        <v>399.99</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Blanc / Guitare</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Noir / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B242" t="n">
-        <v>399.99</v>
+        <v>498.99</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Blanc / Guitare + JW Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Noir / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B243" t="n">
-        <v>474.99</v>
+        <v>499.98</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Donner HUSH X PRO Guitare Électrique - Blanc / Guitare + Pocket Go Pédale</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Blanc / Guitare</t>
         </is>
       </c>
       <c r="B244" t="n">
-        <v>499.98</v>
+        <v>399.99</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Blanc / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B245" t="n">
-        <v>899.99</v>
+        <v>474.99</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano</t>
+          <t>Donner HUSH X PRO Guitare Électrique - Blanc / Guitare + Pocket Go Pédale</t>
         </is>
       </c>
       <c r="B246" t="n">
-        <v>899.99</v>
+        <v>499.98</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc【Pack Officiel】</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2907,7 +2907,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2917,7 +2917,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc【Pack Officiel】</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2927,7 +2927,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc【Pack Officiel】</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2937,337 +2937,337 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Donner Yellow Fall II Pédale 2-en-1 Delay &amp; Reverb</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano</t>
         </is>
       </c>
       <c r="B251" t="n">
-        <v>109.99</v>
+        <v>899.99</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc【Pack Officiel】</t>
         </is>
       </c>
       <c r="B252" t="n">
-        <v>359.99</v>
+        <v>899.99</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano + noir</t>
+          <t>Donner Yellow Fall II Pédale 2-en-1 Delay &amp; Reverb</t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>446.99</v>
+        <v>109.99</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano + banc (match officiel)</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano</t>
         </is>
       </c>
       <c r="B254" t="n">
-        <v>549.98</v>
+        <v>359.99</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano + noir</t>
         </is>
       </c>
       <c r="B255" t="n">
-        <v>584.99</v>
+        <v>446.99</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano + banc (match officiel)</t>
         </is>
       </c>
       <c r="B256" t="n">
-        <v>359.99</v>
+        <v>549.98</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + noir</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B257" t="n">
-        <v>446.99</v>
+        <v>584.99</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + banc (match officiel)</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano</t>
         </is>
       </c>
       <c r="B258" t="n">
-        <v>549.98</v>
+        <v>359.99</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + noir</t>
         </is>
       </c>
       <c r="B259" t="n">
-        <v>584.99</v>
+        <v>446.99</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Donner DED-300X Batterie Electronique</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + banc (match officiel)</t>
         </is>
       </c>
       <c r="B260" t="n">
-        <v>539.99</v>
+        <v>549.98</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Donner DST-80 Débutant Guitare Électrique - Noir</t>
+          <t>【Boîte ouverte】Donner OURA S100 Domestique Piano Numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B261" t="n">
-        <v>130.99</v>
+        <v>584.99</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Donner DST-80 Débutant Guitare Électrique - Sunburst</t>
+          <t>Donner DED-300X Batterie Electronique</t>
         </is>
       </c>
       <c r="B262" t="n">
-        <v>129.99</v>
+        <v>539.99</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano</t>
+          <t>Donner DST-80 Débutant Guitare Électrique - Noir</t>
         </is>
       </c>
       <c r="B263" t="n">
-        <v>659.99</v>
+        <v>130.99</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + banc</t>
+          <t>Donner DST-80 Débutant Guitare Électrique - Sunburst</t>
         </is>
       </c>
       <c r="B264" t="n">
-        <v>782.98</v>
+        <v>129.99</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Banc réglable X-Style</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano</t>
         </is>
       </c>
       <c r="B265" t="n">
-        <v>765.98</v>
+        <v>659.99</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + banc + Tourneur de Page</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + banc</t>
         </is>
       </c>
       <c r="B266" t="n">
-        <v>842.97</v>
+        <v>782.98</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B267" t="n">
-        <v>825.97</v>
+        <v>765.98</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B268" t="n">
-        <v>785.98</v>
+        <v>842.97</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B269" t="n">
-        <v>801.98</v>
+        <v>825.97</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B270" t="n">
-        <v>659.99</v>
+        <v>785.98</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + banc</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Brun foncé / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B271" t="n">
-        <v>765.98</v>
+        <v>801.98</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Banc réglable X-Style</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano</t>
         </is>
       </c>
       <c r="B272" t="n">
-        <v>765.98</v>
+        <v>659.99</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + banc + Tourneur de Page</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + banc</t>
         </is>
       </c>
       <c r="B273" t="n">
-        <v>825.97</v>
+        <v>765.98</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B274" t="n">
-        <v>825.97</v>
+        <v>765.98</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B275" t="n">
-        <v>785.98</v>
+        <v>825.97</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B276" t="n">
-        <v>801.98</v>
+        <v>825.97</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Donner OURA S300 Coussin Épais Banquette Piano (DKB-200 )</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B277" t="n">
-        <v>102.99</v>
+        <v>785.98</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Donner OURA R300 Tabouret assorti avec Coussin Épais (DKB-300) - couleur bois clair</t>
+          <t>Donner DDP-200 PRO Pondéré à Marteau Piano Numérique - Noir / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B278" t="n">
-        <v>92.98999999999999</v>
+        <v>801.98</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Donner OURA R300 Tabouret assorti avec Coussin Épais (DKB-300) - couleur noyer</t>
+          <t>Donner OURA S300 Coussin Épais Banquette Piano (DKB-200 )</t>
         </is>
       </c>
       <c r="B279" t="n">
-        <v>109.99</v>
+        <v>102.99</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Donner Triple Threat 3-en-1 Pédale Guitare</t>
+          <t>Donner OURA R300 Tabouret assorti avec Coussin Épais (DKB-300) - couleur bois clair</t>
         </is>
       </c>
       <c r="B280" t="n">
-        <v>99</v>
+        <v>92.98999999999999</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Donner DT-50 Tabouret de Batterie</t>
+          <t>Donner OURA R300 Tabouret assorti avec Coussin Épais (DKB-300) - couleur noyer</t>
         </is>
       </c>
       <c r="B281" t="n">
-        <v>72.98999999999999</v>
+        <v>109.99</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Donner DST-550 Guitare Électrique - Bleu</t>
+          <t>Donner Triple Threat 3-en-1 Pédale Guitare</t>
         </is>
       </c>
       <c r="B282" t="n">
-        <v>169.99</v>
+        <v>99</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Donner DST-550 Guitare Électrique - Littoral caribéen Gradation LR</t>
+          <t>Donner DT-50 Tabouret de Batterie</t>
         </is>
       </c>
       <c r="B283" t="n">
-        <v>199.99</v>
+        <v>72.98999999999999</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Donner DST-550 Guitare Électrique - Blanc</t>
+          <t>Donner DST-550 Guitare Électrique - Bleu</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -3277,1737 +3277,1737 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Noir / Piano</t>
+          <t>Donner DST-550 Guitare Électrique - Littoral caribéen Gradation LR</t>
         </is>
       </c>
       <c r="B285" t="n">
-        <v>289.99</v>
+        <v>199.99</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Noir / Piano + Banc Noir</t>
+          <t>Donner DST-550 Guitare Électrique - Blanc</t>
         </is>
       </c>
       <c r="B286" t="n">
-        <v>379.98</v>
+        <v>169.99</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Rouge / Piano</t>
+          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Noir / Piano</t>
         </is>
       </c>
       <c r="B287" t="n">
-        <v>279.99</v>
+        <v>289.99</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Rouge / Piano + Banc Noir</t>
+          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Noir / Piano + Banc Noir</t>
         </is>
       </c>
       <c r="B288" t="n">
-        <v>409.98</v>
+        <v>379.98</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Donner DDP-95 lesté Piano numérique - Blanc / Piano</t>
+          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Rouge / Piano</t>
         </is>
       </c>
       <c r="B289" t="n">
-        <v>389.99</v>
+        <v>279.99</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Donner DDP-95 lesté Piano numérique - Blanc / Piano + banc de piano</t>
+          <t>Donner DEP-16S Piano Numérique en Acier Lesté - Rouge / Piano + Banc Noir</t>
         </is>
       </c>
       <c r="B290" t="n">
-        <v>495.98</v>
+        <v>409.98</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Donner DDP-95 lesté Piano numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-95 lesté Piano numérique - Blanc / Piano</t>
         </is>
       </c>
       <c r="B291" t="n">
-        <v>519.98</v>
+        <v>389.99</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Donner DDP-95 lesté Piano numérique - Noir / Piano</t>
+          <t>Donner DDP-95 lesté Piano numérique - Blanc / Piano + banc de piano</t>
         </is>
       </c>
       <c r="B292" t="n">
-        <v>389.99</v>
+        <v>495.98</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Donner DDP-95 lesté Piano numérique - Noir / Piano + banc de piano</t>
+          <t>Donner DDP-95 lesté Piano numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B293" t="n">
-        <v>479.98</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Donner DDP-95 lesté Piano numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-95 lesté Piano numérique - Noir / Piano</t>
         </is>
       </c>
       <c r="B294" t="n">
-        <v>519.98</v>
+        <v>389.99</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano</t>
+          <t>Donner DDP-95 lesté Piano numérique - Noir / Piano + banc de piano</t>
         </is>
       </c>
       <c r="B295" t="n">
-        <v>209.99</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc réglable X-Style</t>
+          <t>Donner DDP-95 lesté Piano numérique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B296" t="n">
-        <v>284.99</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano Marron</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano</t>
         </is>
       </c>
       <c r="B297" t="n">
-        <v>315.98</v>
+        <v>209.99</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B298" t="n">
-        <v>309.98</v>
+        <v>284.99</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B299" t="n">
-        <v>359.97</v>
+        <v>315.98</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B300" t="n">
-        <v>385.97</v>
+        <v>309.98</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B301" t="n">
-        <v>379.97</v>
+        <v>359.97</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B302" t="n">
-        <v>319.98</v>
+        <v>385.97</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B303" t="n">
-        <v>389.97</v>
+        <v>379.97</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B304" t="n">
-        <v>179.99</v>
+        <v>319.98</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc réglable X-Style</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel【Nouvelle version】 / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B305" t="n">
-        <v>259.98</v>
+        <v>389.97</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano Marron</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano</t>
         </is>
       </c>
       <c r="B306" t="n">
-        <v>267.98</v>
+        <v>179.99</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B307" t="n">
-        <v>276.98</v>
+        <v>259.98</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B308" t="n">
-        <v>319.97</v>
+        <v>267.98</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B309" t="n">
-        <v>327.97</v>
+        <v>276.98</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B310" t="n">
-        <v>336.97</v>
+        <v>319.97</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B311" t="n">
-        <v>279.98</v>
+        <v>327.97</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B312" t="n">
-        <v>339.97</v>
+        <v>336.97</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B313" t="n">
-        <v>189.99</v>
+        <v>279.98</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc réglable X-Style</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois naturel / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B314" t="n">
-        <v>265.98</v>
+        <v>339.97</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano Marron</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano</t>
         </is>
       </c>
       <c r="B315" t="n">
-        <v>273.98</v>
+        <v>189.99</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B316" t="n">
-        <v>282.98</v>
+        <v>265.98</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B317" t="n">
-        <v>335.97</v>
+        <v>273.98</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B318" t="n">
-        <v>343.97</v>
+        <v>282.98</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B319" t="n">
-        <v>352.97</v>
+        <v>335.97</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B320" t="n">
-        <v>285.98</v>
+        <v>343.97</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B321" t="n">
-        <v>355.97</v>
+        <v>352.97</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B322" t="n">
-        <v>209.99</v>
+        <v>285.98</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc réglable X-Style</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - couleur bois clair / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B323" t="n">
-        <v>289.98</v>
+        <v>355.97</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano Marron</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano</t>
         </is>
       </c>
       <c r="B324" t="n">
-        <v>315.98</v>
+        <v>209.99</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc réglable X-Style</t>
         </is>
       </c>
       <c r="B325" t="n">
-        <v>309.98</v>
+        <v>289.98</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc réglable X-Style + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B326" t="n">
-        <v>359.97</v>
+        <v>315.98</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B327" t="n">
-        <v>385.97</v>
+        <v>309.98</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc réglable X-Style + Tourneur de Page</t>
         </is>
       </c>
       <c r="B328" t="n">
-        <v>379.97</v>
+        <v>359.97</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B329" t="n">
-        <v>319.98</v>
+        <v>385.97</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B330" t="n">
-        <v>389.97</v>
+        <v>379.97</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Donner DP-10 Portable Pliable Piano Numerique - Piano</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B331" t="n">
-        <v>169.99</v>
+        <v>319.98</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Donner DP-10 Portable Pliable Piano Numerique - Piano + Banc</t>
+          <t>Donner DEP-1S Semi-Lesté De Style Bois Piano Numérique - brun antique / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B332" t="n">
-        <v>239.98</v>
+        <v>389.97</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Noir Space Fly / Guitare</t>
+          <t>Donner DP-10 Portable Pliable Piano Numerique - Piano</t>
         </is>
       </c>
       <c r="B333" t="n">
-        <v>359.99</v>
+        <v>169.99</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Noir Space Fly / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DP-10 Portable Pliable Piano Numerique - Piano + Banc</t>
         </is>
       </c>
       <c r="B334" t="n">
-        <v>559.99</v>
+        <v>239.98</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Noir Space Fly / Guitare + JW Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Noir Space Fly / Guitare</t>
         </is>
       </c>
       <c r="B335" t="n">
-        <v>458.99</v>
+        <v>359.99</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Blanc / Guitare</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Noir Space Fly / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B336" t="n">
-        <v>309.99</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Blanc / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Noir Space Fly / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B337" t="n">
-        <v>559.99</v>
+        <v>458.99</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Blanc / Guitare + JW Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Blanc / Guitare</t>
         </is>
       </c>
       <c r="B338" t="n">
-        <v>458.99</v>
+        <v>309.99</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Bleu Hawaï / Guitare</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Blanc / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B339" t="n">
-        <v>359.99</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Bleu Hawaï / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Blanc / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B340" t="n">
-        <v>559.99</v>
+        <v>458.99</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Bleu Hawaï / Guitare + JW Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Bleu Hawaï / Guitare</t>
         </is>
       </c>
       <c r="B341" t="n">
-        <v>458.99</v>
+        <v>359.99</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Marron Dégradé Maillard / Guitare</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Bleu Hawaï / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B342" t="n">
-        <v>359.99</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Marron Dégradé Maillard / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Bleu Hawaï / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B343" t="n">
-        <v>559.99</v>
+        <v>458.99</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Marron Dégradé Maillard / Guitare + JW Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Marron Dégradé Maillard / Guitare</t>
         </is>
       </c>
       <c r="B344" t="n">
-        <v>458.99</v>
+        <v>359.99</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Sunburst / Guitare</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Marron Dégradé Maillard / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B345" t="n">
-        <v>309.99</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Sunburst / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Marron Dégradé Maillard / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B346" t="n">
-        <v>559.99</v>
+        <v>458.99</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Sunburst / Guitare + JW Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Sunburst / Guitare</t>
         </is>
       </c>
       <c r="B347" t="n">
-        <v>458.99</v>
+        <v>309.99</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Naturel / Guitare</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Sunburst / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B348" t="n">
-        <v>309.99</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Naturel / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Sunburst / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B349" t="n">
-        <v>559.99</v>
+        <v>458.99</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Naturel / Guitare + JW Pédale</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Naturel / Guitare</t>
         </is>
       </c>
       <c r="B350" t="n">
-        <v>458.99</v>
+        <v>309.99</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Donner DED-200 Max Batteries Electroniques</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Naturel / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B351" t="n">
-        <v>499.99</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Donner BackBeat Batterie Electronique - BackBeat</t>
+          <t>Donner HUSH I PRO Electro-Acoustique Guitare Voyageuse - Naturel / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B352" t="n">
-        <v>1099.99</v>
+        <v>458.99</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Donner BackBeat Batterie Electronique - BackBeat + Tabouret de batterie DT-50</t>
+          <t>Donner DED-200 Max Batteries Electroniques</t>
         </is>
       </c>
       <c r="B353" t="n">
-        <v>1114.99</v>
+        <v>499.99</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Pro Rétro esthétique Piano Numérique - DDP-80 Pro Piano</t>
+          <t>Donner BackBeat Batterie Electronique - BackBeat</t>
         </is>
       </c>
       <c r="B354" t="n">
-        <v>899</v>
+        <v>1099.99</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Pro Rétro esthétique Piano Numérique - Piano + Banc de Piano</t>
+          <t>Donner BackBeat Batterie Electronique - BackBeat + Tabouret de batterie DT-50</t>
         </is>
       </c>
       <c r="B355" t="n">
-        <v>995.99</v>
+        <v>1114.99</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Pro Rétro esthétique Piano Numérique - Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-80 Pro Rétro esthétique Piano Numérique - DDP-80 Pro Piano</t>
         </is>
       </c>
       <c r="B356" t="n">
-        <v>998.99</v>
+        <v>899</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Donner DAG-1CB Débutant Guitare Acoustique - Dreadnought Cutaway</t>
+          <t>Donner DDP-80 Pro Rétro esthétique Piano Numérique - Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B357" t="n">
-        <v>125.99</v>
+        <v>995.99</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>Donner DAG-1CB Débutant Guitare Acoustique - Dreadnought</t>
+          <t>Donner DDP-80 Pro Rétro esthétique Piano Numérique - Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B358" t="n">
-        <v>166.99</v>
+        <v>998.99</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - naturel / Guitare</t>
+          <t>Donner DAG-1CB Débutant Guitare Acoustique - Dreadnought Cutaway</t>
         </is>
       </c>
       <c r="B359" t="n">
-        <v>299.99</v>
+        <v>125.99</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - naturel / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DAG-1CB Débutant Guitare Acoustique - Dreadnought</t>
         </is>
       </c>
       <c r="B360" t="n">
-        <v>536.98</v>
+        <v>166.99</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - naturel / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - naturel / Guitare</t>
         </is>
       </c>
       <c r="B361" t="n">
-        <v>448.99</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - naturel / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B362" t="n">
-        <v>299.99</v>
+        <v>536.98</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - naturel / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B363" t="n">
-        <v>536.98</v>
+        <v>448.99</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare</t>
         </is>
       </c>
       <c r="B364" t="n">
-        <v>448.99</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B365" t="n">
-        <v>299.99</v>
+        <v>536.98</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B366" t="n">
-        <v>536.98</v>
+        <v>448.99</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare</t>
         </is>
       </c>
       <c r="B367" t="n">
-        <v>448.99</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B368" t="n">
-        <v>299.99</v>
+        <v>536.98</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B369" t="n">
-        <v>536.98</v>
+        <v>448.99</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare</t>
         </is>
       </c>
       <c r="B370" t="n">
-        <v>448.99</v>
+        <v>299.99</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>Donner Bois Massif Banc Piano avec Rangement</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B371" t="n">
-        <v>109.99</v>
+        <v>536.98</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B372" t="n">
-        <v>319.99</v>
+        <v>448.99</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc de Piano bois clair</t>
+          <t>Donner Bois Massif Banc Piano avec Rangement</t>
         </is>
       </c>
       <c r="B373" t="n">
-        <v>408.99</v>
+        <v>109.99</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc de Piano Blanc</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano</t>
         </is>
       </c>
       <c r="B374" t="n">
-        <v>425.98</v>
+        <v>319.99</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc de Piano bois clair</t>
         </is>
       </c>
       <c r="B375" t="n">
-        <v>417.98</v>
+        <v>408.99</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc réglable en hauteur</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc de Piano Blanc</t>
         </is>
       </c>
       <c r="B376" t="n">
-        <v>429.98</v>
+        <v>425.98</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B377" t="n">
-        <v>489.97</v>
+        <v>417.98</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc Duo réglable en hauteur</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B378" t="n">
-        <v>445.98</v>
+        <v>429.98</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B379" t="n">
-        <v>505.97</v>
+        <v>489.97</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Beige mat Banc réglable en hauteur</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc Duo réglable en hauteur</t>
         </is>
       </c>
       <c r="B380" t="n">
-        <v>449.98</v>
+        <v>445.98</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B381" t="n">
-        <v>329.99</v>
+        <v>505.97</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc de Piano bois clair</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Bois clair / Piano + Beige mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B382" t="n">
-        <v>428.98</v>
+        <v>449.98</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc de Piano Blanc</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano</t>
         </is>
       </c>
       <c r="B383" t="n">
-        <v>425.98</v>
+        <v>329.99</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc de Piano bois clair</t>
         </is>
       </c>
       <c r="B384" t="n">
-        <v>417.98</v>
+        <v>428.98</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc réglable en hauteur</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc de Piano Blanc</t>
         </is>
       </c>
       <c r="B385" t="n">
-        <v>429.98</v>
+        <v>425.98</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B386" t="n">
-        <v>489.97</v>
+        <v>417.98</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc Duo réglable en hauteur</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B387" t="n">
-        <v>445.98</v>
+        <v>429.98</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B388" t="n">
-        <v>505.97</v>
+        <v>489.97</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Beige mat Banc réglable en hauteur</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc Duo réglable en hauteur</t>
         </is>
       </c>
       <c r="B389" t="n">
-        <v>449.98</v>
+        <v>445.98</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - DDP-80 PLUS Piano</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B390" t="n">
-        <v>499.99</v>
+        <v>505.97</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-60 Semi-lesté Piano Numérique - Gris-brun / Piano + Beige mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B391" t="n">
-        <v>627.98</v>
+        <v>449.98</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - DDP-80 PLUS Piano</t>
         </is>
       </c>
       <c r="B392" t="n">
-        <v>636.98</v>
+        <v>499.99</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B393" t="n">
-        <v>697.97</v>
+        <v>627.98</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B394" t="n">
-        <v>706.97</v>
+        <v>636.98</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Höhenverstellbarer banc</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B395" t="n">
-        <v>639.98</v>
+        <v>697.97</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B396" t="n">
-        <v>699.97</v>
+        <v>706.97</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B397" t="n">
-        <v>655.98</v>
+        <v>639.98</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B398" t="n">
-        <v>715.97</v>
+        <v>699.97</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B399" t="n">
-        <v>659.98</v>
+        <v>655.98</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B400" t="n">
-        <v>499.99</v>
+        <v>715.97</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Banc X-Style</t>
+          <t>Donner DDP-80 PLUS Piano Numérique Avec Couvercle Semi-Ouvert - Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B401" t="n">
-        <v>579.99</v>
+        <v>659.98</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Banc de Piano</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano</t>
         </is>
       </c>
       <c r="B402" t="n">
-        <v>579.98</v>
+        <v>499.99</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Banc X-Style</t>
         </is>
       </c>
       <c r="B403" t="n">
-        <v>639.97</v>
+        <v>579.99</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Duo Höhenverstellbarer banc</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B404" t="n">
-        <v>615.98</v>
+        <v>579.98</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B405" t="n">
-        <v>675.97</v>
+        <v>639.97</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Höhenverstellbarer banc</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B406" t="n">
-        <v>599.98</v>
+        <v>615.98</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B407" t="n">
-        <v>659.97</v>
+        <v>675.97</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B408" t="n">
-        <v>619.98</v>
+        <v>599.98</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B409" t="n">
-        <v>459.99</v>
+        <v>659.97</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Banc X-Style</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 Pro / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B410" t="n">
-        <v>539.99</v>
+        <v>619.98</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Banc de Piano</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano</t>
         </is>
       </c>
       <c r="B411" t="n">
-        <v>579.98</v>
+        <v>459.99</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Banc X-Style</t>
         </is>
       </c>
       <c r="B412" t="n">
-        <v>639.97</v>
+        <v>539.99</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Duo Höhenverstellbarer banc</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B413" t="n">
-        <v>605.98</v>
+        <v>579.98</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B414" t="n">
-        <v>665.97</v>
+        <v>639.97</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano numérique</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B415" t="n">
-        <v>629.99</v>
+        <v>605.98</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano +  Tabouret de piano blanc</t>
+          <t>【Déstockage】Donner DDP-90 PRO Domestique Piano Numérique - DDP-90 / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B416" t="n">
-        <v>825.98</v>
+        <v>665.97</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano numérique</t>
         </is>
       </c>
       <c r="B417" t="n">
-        <v>895.97</v>
+        <v>629.99</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano +  Tabouret de piano noir</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano +  Tabouret de piano blanc</t>
         </is>
       </c>
       <c r="B418" t="n">
-        <v>809.98</v>
+        <v>825.98</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B419" t="n">
-        <v>845.98</v>
+        <v>895.97</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano +  Tabouret de piano noir</t>
         </is>
       </c>
       <c r="B420" t="n">
-        <v>849.98</v>
+        <v>809.98</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano numérique</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B421" t="n">
-        <v>761.75</v>
+        <v>845.98</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano +  Tabouret de piano blanc</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B422" t="n">
-        <v>851.4299999999999</v>
+        <v>849.98</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano numérique</t>
         </is>
       </c>
       <c r="B423" t="n">
-        <v>927.86</v>
+        <v>761.75</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano +  Tabouret de piano noir</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano +  Tabouret de piano blanc</t>
         </is>
       </c>
       <c r="B424" t="n">
-        <v>840.65</v>
+        <v>851.4299999999999</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B425" t="n">
-        <v>977.62</v>
+        <v>927.86</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano Numérique</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano +  Tabouret de piano noir</t>
         </is>
       </c>
       <c r="B426" t="n">
-        <v>629.99</v>
+        <v>840.65</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Banc de Piano</t>
+          <t>Donner DDP-100 Vertical lesté Piano Numérique - Noir / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B427" t="n">
-        <v>787.98</v>
+        <v>977.62</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano Numérique</t>
         </is>
       </c>
       <c r="B428" t="n">
-        <v>857.97</v>
+        <v>629.99</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B429" t="n">
-        <v>799.98</v>
+        <v>787.98</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B430" t="n">
-        <v>859.97</v>
+        <v>857.97</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B431" t="n">
-        <v>815.98</v>
+        <v>799.98</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B432" t="n">
-        <v>875.97</v>
+        <v>859.97</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano Numérique</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B433" t="n">
-        <v>559.99</v>
+        <v>815.98</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Banc de Piano</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 MK2【Son amélioré】 / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B434" t="n">
-        <v>737.98</v>
+        <v>875.97</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano Numérique</t>
         </is>
       </c>
       <c r="B435" t="n">
-        <v>807.97</v>
+        <v>559.99</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B436" t="n">
-        <v>749.98</v>
+        <v>737.98</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B437" t="n">
-        <v>809.97</v>
+        <v>807.97</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Duo Höhenverstellbarer banc</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B438" t="n">
-        <v>765.98</v>
+        <v>749.98</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B439" t="n">
-        <v>825.97</v>
+        <v>809.97</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>Donner Arena 2000 Pédale Multi-Effets Guitare - Arena 2000</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Duo Höhenverstellbarer banc</t>
         </is>
       </c>
       <c r="B440" t="n">
-        <v>186.99</v>
+        <v>765.98</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>Donner DKB-10 Bois Massif Banc Piano avec Rangement - Marron</t>
+          <t>Donner DDP-200 MK2 Piano numérique avec mécanisme de marteau gradué - DDP-200 / Piano + Duo Höhenverstellbarer banc + Tourneur de Page</t>
         </is>
       </c>
       <c r="B441" t="n">
-        <v>99.98999999999999</v>
+        <v>825.97</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>Donner DKB-10 Bois Massif Banc Piano avec Rangement - Blanc</t>
+          <t>Donner Arena 2000 Pédale Multi-Effets Guitare - Arena 2000</t>
         </is>
       </c>
       <c r="B442" t="n">
-        <v>99.98999999999999</v>
+        <v>186.99</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>Donner DMK-25 Pro Clavier MIDI</t>
+          <t>Donner DKB-10 Bois Massif Banc Piano avec Rangement - Marron</t>
         </is>
       </c>
       <c r="B443" t="n">
-        <v>89.98999999999999</v>
+        <v>99.98999999999999</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Rouge / Guitare</t>
+          <t>Donner DKB-10 Bois Massif Banc Piano avec Rangement - Blanc</t>
         </is>
       </c>
       <c r="B444" t="n">
-        <v>236.99</v>
+        <v>99.98999999999999</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Rouge / Guitare + JW Pédale</t>
+          <t>Donner DMK-25 Pro Clavier MIDI</t>
         </is>
       </c>
       <c r="B445" t="n">
-        <v>370.99</v>
+        <v>89.98999999999999</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Rouge / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Rouge / Guitare</t>
         </is>
       </c>
       <c r="B446" t="n">
-        <v>491.98</v>
+        <v>236.99</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Noir / Guitare</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Rouge / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B447" t="n">
-        <v>219.99</v>
+        <v>370.99</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Noir / Guitare + JW Pédale</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Rouge / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B448" t="n">
-        <v>370.99</v>
+        <v>491.98</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Noir / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Noir / Guitare</t>
         </is>
       </c>
       <c r="B449" t="n">
-        <v>491.98</v>
+        <v>219.99</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Marron / Guitare</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Noir / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B450" t="n">
-        <v>281.99</v>
+        <v>370.99</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Marron / Guitare + JW Pédale</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Noir / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B451" t="n">
-        <v>373.37</v>
+        <v>491.98</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Marron / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Marron / Guitare</t>
         </is>
       </c>
       <c r="B452" t="n">
-        <v>530.16</v>
+        <v>281.99</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>Donner Essential B1 Synthétiseur de basse analogique - B1</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Marron / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B453" t="n">
-        <v>89</v>
+        <v>373.37</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>Donner Bois Massif Banc Piano avec Rangement</t>
+          <t>Donner DJP-1000 Guitare Jazz Demi-Caisse - Marron / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B454" t="n">
-        <v>109.99</v>
+        <v>530.16</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>Pour la différence de prix</t>
+          <t>Donner Essential B1 Synthétiseur de basse analogique - B1</t>
         </is>
       </c>
       <c r="B455" t="n">
-        <v>7.69</v>
+        <v>89</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Bleu / Guitare</t>
+          <t>Donner Bois Massif Banc Piano avec Rangement</t>
         </is>
       </c>
       <c r="B456" t="n">
-        <v>152.99</v>
+        <v>109.99</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Bleu / Guitare + Arena 2000 Pédale</t>
+          <t>Pour la différence de prix</t>
         </is>
       </c>
       <c r="B457" t="n">
-        <v>352.99</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Ivoire Blanc / Guitare</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Bleu / Guitare</t>
         </is>
       </c>
       <c r="B458" t="n">
@@ -5017,7 +5017,7 @@
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Ivoire Blanc / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Bleu / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B459" t="n">
@@ -5027,7 +5027,7 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Sunburst / Guitare</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Ivoire Blanc / Guitare</t>
         </is>
       </c>
       <c r="B460" t="n">
@@ -5037,7 +5037,7 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Sunburst / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Ivoire Blanc / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B461" t="n">
@@ -5047,7 +5047,7 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Noir / Guitare</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Sunburst / Guitare</t>
         </is>
       </c>
       <c r="B462" t="n">
@@ -5057,7 +5057,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Noir / Guitare + Arena 2000 Pédale</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Sunburst / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B463" t="n">
@@ -5067,147 +5067,147 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>Donner DBM-10 Bluetooth Auto  Sans Fil Page Turner Pédale - Noir</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Noir / Guitare</t>
         </is>
       </c>
       <c r="B464" t="n">
-        <v>86.98999999999999</v>
+        <v>152.99</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>Donner DBM-10 Bluetooth Auto  Sans Fil Page Turner Pédale - Argent</t>
+          <t>Donner DST-152 Guitare Électrique avec Ampli et Housse - Noir / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B465" t="n">
-        <v>69.98999999999999</v>
+        <v>352.99</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano</t>
+          <t>Donner DBM-10 Bluetooth Auto  Sans Fil Page Turner Pédale - Noir</t>
         </is>
       </c>
       <c r="B466" t="n">
-        <v>389.99</v>
+        <v>86.98999999999999</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Banc X-Style</t>
+          <t>Donner DBM-10 Bluetooth Auto  Sans Fil Page Turner Pédale - Argent</t>
         </is>
       </c>
       <c r="B467" t="n">
-        <v>479.98</v>
+        <v>69.98999999999999</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Tabouret de piano noir</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano</t>
         </is>
       </c>
       <c r="B468" t="n">
-        <v>479.98</v>
+        <v>389.99</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Tabouret de piano blanc</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Banc X-Style</t>
         </is>
       </c>
       <c r="B469" t="n">
-        <v>495.98</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Tabouret de piano noir</t>
         </is>
       </c>
       <c r="B470" t="n">
-        <v>519.98</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Tabouret de piano blanc</t>
         </is>
       </c>
       <c r="B471" t="n">
-        <v>399.99</v>
+        <v>495.98</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Banc X-Style</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Noir / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B472" t="n">
-        <v>479.98</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Tabouret de piano noir</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano</t>
         </is>
       </c>
       <c r="B473" t="n">
-        <v>479.98</v>
+        <v>399.99</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Tabouret de piano blanc</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Banc X-Style</t>
         </is>
       </c>
       <c r="B474" t="n">
-        <v>495.98</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Tabouret de piano noir</t>
         </is>
       </c>
       <c r="B475" t="n">
-        <v>519.98</v>
+        <v>479.98</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>Donner Tabouret de piano en forme de X réglable en hauteur - 15.7*11.8*2.4pouces</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Tabouret de piano blanc</t>
         </is>
       </c>
       <c r="B476" t="n">
-        <v>89.98999999999999</v>
+        <v>495.98</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>Donner Tabouret de piano en forme de X réglable en hauteur - 15.7*11.8*1.6pouces</t>
+          <t>Donner DEP-20 lestées Piano Numerique - Blanc / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B477" t="n">
-        <v>79.47</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>Donner Bois Massif Banc Piano avec Rangement</t>
+          <t>Donner Tabouret de piano en forme de X réglable en hauteur - 15.7*11.8*2.4pouces</t>
         </is>
       </c>
       <c r="B478" t="n">
@@ -5217,480 +5217,500 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / DDP-80</t>
+          <t>Donner Tabouret de piano en forme de X réglable en hauteur - 15.7*11.8*1.6pouces</t>
         </is>
       </c>
       <c r="B479" t="n">
-        <v>469.99</v>
+        <v>79.47</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Casque audio M100</t>
+          <t>Donner Bois Massif Banc Piano avec Rangement</t>
         </is>
       </c>
       <c r="B480" t="n">
-        <v>518.99</v>
+        <v>89.98999999999999</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / DDP-80</t>
         </is>
       </c>
       <c r="B481" t="n">
-        <v>566.98</v>
+        <v>469.99</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Casque audio M100</t>
         </is>
       </c>
       <c r="B482" t="n">
-        <v>557.98</v>
+        <v>518.99</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B483" t="n">
-        <v>636.97</v>
+        <v>566.98</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B484" t="n">
-        <v>627.97</v>
+        <v>557.98</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano Noir</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B485" t="n">
-        <v>549.98</v>
+        <v>636.97</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B486" t="n">
-        <v>569.98</v>
+        <v>627.97</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc de Piano Noir</t>
         </is>
       </c>
       <c r="B487" t="n">
-        <v>629.97</v>
+        <v>549.98</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc Duo réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B488" t="n">
-        <v>585.98</v>
+        <v>569.98</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B489" t="n">
-        <v>645.97</v>
+        <v>629.97</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc Duo réglable en hauteur</t>
         </is>
       </c>
       <c r="B490" t="n">
-        <v>589.98</v>
+        <v>585.98</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / DDP-80</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B491" t="n">
-        <v>429.99</v>
+        <v>645.97</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Casque audio M100</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Son amélioré / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B492" t="n">
-        <v>489.99</v>
+        <v>589.98</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / DDP-80</t>
         </is>
       </c>
       <c r="B493" t="n">
-        <v>536.98</v>
+        <v>429.99</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Casque audio M100</t>
         </is>
       </c>
       <c r="B494" t="n">
-        <v>527.98</v>
+        <v>489.99</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B495" t="n">
-        <v>606.97</v>
+        <v>536.98</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B496" t="n">
-        <v>597.97</v>
+        <v>527.98</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano Noir</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B497" t="n">
-        <v>519.98</v>
+        <v>606.97</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B498" t="n">
-        <v>539.98</v>
+        <v>597.97</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc de Piano Noir</t>
         </is>
       </c>
       <c r="B499" t="n">
-        <v>599.97</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc Duo réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B500" t="n">
-        <v>555.98</v>
+        <v>539.98</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B501" t="n">
-        <v>615.97</v>
+        <v>599.97</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc Duo réglable en hauteur</t>
         </is>
       </c>
       <c r="B502" t="n">
-        <v>559.98</v>
+        <v>555.98</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / DDP-80</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B503" t="n">
-        <v>469.99</v>
+        <v>615.97</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Casque audio M100</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Bois naturel / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B504" t="n">
-        <v>529.99</v>
+        <v>559.98</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / DDP-80</t>
         </is>
       </c>
       <c r="B505" t="n">
-        <v>566.98</v>
+        <v>469.99</v>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Casque audio M100</t>
         </is>
       </c>
       <c r="B506" t="n">
-        <v>557.98</v>
+        <v>529.99</v>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B507" t="n">
-        <v>636.97</v>
+        <v>566.98</v>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B508" t="n">
-        <v>627.97</v>
+        <v>557.98</v>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano Noir</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B509" t="n">
-        <v>549.98</v>
+        <v>636.97</v>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B510" t="n">
-        <v>569.98</v>
+        <v>627.97</v>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc de Piano Noir</t>
         </is>
       </c>
       <c r="B511" t="n">
-        <v>629.97</v>
+        <v>549.98</v>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc Duo réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B512" t="n">
-        <v>585.98</v>
+        <v>569.98</v>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B513" t="n">
-        <v>645.97</v>
+        <v>629.97</v>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Blanc mat Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc Duo réglable en hauteur</t>
         </is>
       </c>
       <c r="B514" t="n">
-        <v>589.98</v>
+        <v>585.98</v>
       </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / DDP-80</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B515" t="n">
-        <v>429.99</v>
+        <v>645.97</v>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Casque audio M100</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer【Son amélioré】 / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B516" t="n">
-        <v>499.99</v>
+        <v>589.98</v>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / DDP-80</t>
         </is>
       </c>
       <c r="B517" t="n">
-        <v>536.98</v>
+        <v>429.99</v>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano Marron</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Casque audio M100</t>
         </is>
       </c>
       <c r="B518" t="n">
-        <v>527.98</v>
+        <v>499.99</v>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano</t>
         </is>
       </c>
       <c r="B519" t="n">
-        <v>606.97</v>
+        <v>536.98</v>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano Marron + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano Marron</t>
         </is>
       </c>
       <c r="B520" t="n">
-        <v>597.97</v>
+        <v>527.98</v>
       </c>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano Noir</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano + Tourneur de Page</t>
         </is>
       </c>
       <c r="B521" t="n">
-        <v>519.98</v>
+        <v>606.97</v>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano Marron + Tourneur de Page</t>
         </is>
       </c>
       <c r="B522" t="n">
-        <v>539.98</v>
+        <v>597.97</v>
       </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc de Piano Noir</t>
         </is>
       </c>
       <c r="B523" t="n">
-        <v>599.97</v>
+        <v>519.98</v>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc Duo réglable en hauteur</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc réglable en hauteur</t>
         </is>
       </c>
       <c r="B524" t="n">
-        <v>555.98</v>
+        <v>539.98</v>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc réglable en hauteur + Tourneur de Page</t>
         </is>
       </c>
       <c r="B525" t="n">
-        <v>615.97</v>
+        <v>599.97</v>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc Duo réglable en hauteur</t>
+        </is>
+      </c>
+      <c r="B526" t="n">
+        <v>555.98</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Banc Duo réglable en hauteur + Tourneur de Page</t>
+        </is>
+      </c>
+      <c r="B527" t="n">
+        <v>615.97</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
           <t>Donner DDP-80 Motif de Bois Piano Numérique - Noyer / Piano + Blanc mat Banc réglable en hauteur</t>
         </is>
       </c>
-      <c r="B526" t="n">
+      <c r="B528" t="n">
         <v>559.98</v>
       </c>
     </row>

</xml_diff>